<commit_message>
Completed the debug for Nebula-Galaxy.
Next: Working on changing the 0 and 1 into False and True
</commit_message>
<xml_diff>
--- a/SWTest/Outputs/Navigator_Analysis_20250806_114628.xlsx
+++ b/SWTest/Outputs/Navigator_Analysis_20250806_114628.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45A4FF9-1763-473B-A8B6-1A4E1B17DFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA5825E6-F8E2-453B-AA13-B89C0EC366AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28695" yWindow="-6795" windowWidth="16410" windowHeight="9465" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -964,7 +964,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -976,6 +976,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1013,13 +1019,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1372,7 +1381,7 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">

</xml_diff>